<commit_message>
Fix Cloudflare Pages build v3.2.4
</commit_message>
<xml_diff>
--- a/templates/SubsTracker_订阅批量导入模板.xlsx
+++ b/templates/SubsTracker_订阅批量导入模板.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="订阅导入模板" sheetId="1" r:id="Rd91b3834e0c741ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R6aeb36c61f274010"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选项" sheetId="3" r:id="Rfc3264e5e8714e22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="订阅导入模板" sheetId="1" r:id="Rc4ba49667ad04770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="Rbb7790b842144282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选项" sheetId="3" r:id="Rfc87dfb107324cdf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -43,8 +43,13 @@
       <x:color rgb="FF374151"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -66,81 +71,38 @@
         <x:fgColor rgb="FFF9FAFB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="20">
     <x:border/>
     <x:border/>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="72">
+  <x:cellXfs count="76">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -324,6 +286,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -5266,8 +5234,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -5468,9 +5438,62 @@
         <x:v>自由文本。</x:v>
       </x:c>
     </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="75" t="str">
+        <x:v>v3.2.8 导入规则</x:v>
+      </x:c>
+      <x:c r="B27" s="75" t="str"/>
+      <x:c r="C27" s="75" t="str"/>
+      <x:c r="D27" s="75" t="str"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="12" t="str">
+        <x:v>Excel 文件直接导入</x:v>
+      </x:c>
+      <x:c r="B28" s="12" t="str"/>
+      <x:c r="C28" s="12" t="str">
+        <x:v>支持 .xlsx / .xls / .csv / .tsv，也支持从 Excel 复制粘贴。</x:v>
+      </x:c>
+      <x:c r="D28" s="12" t="str"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="12" t="str">
+        <x:v>只新增、不覆盖</x:v>
+      </x:c>
+      <x:c r="B29" s="12" t="str"/>
+      <x:c r="C29" s="12" t="str">
+        <x:v>导入不会更新或覆盖已有订阅；检测到原有记录会自动跳过并在结果中报告。</x:v>
+      </x:c>
+      <x:c r="D29" s="12" t="str"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="12" t="str">
+        <x:v>批量操作</x:v>
+      </x:c>
+      <x:c r="B30" s="12" t="str"/>
+      <x:c r="C30" s="12" t="str">
+        <x:v>导入前可预览；错误行不会阻断其他有效数据。</x:v>
+      </x:c>
+      <x:c r="D30" s="12" t="str"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="12" t="str">
+        <x:v>账号密码</x:v>
+      </x:c>
+      <x:c r="B31" s="12" t="str"/>
+      <x:c r="C31" s="12" t="str">
+        <x:v>订阅导入不包含密码；密码仍由 Database 账号库独立管理。</x:v>
+      </x:c>
+      <x:c r="D31" s="12" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:B1"/>
+    <x:mergeCell ref="A27:D27"/>
+    <x:mergeCell ref="A28:D28"/>
+    <x:mergeCell ref="A29:D29"/>
+    <x:mergeCell ref="A30:D30"/>
+    <x:mergeCell ref="A31:D31"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>